<commit_message>
chore: update IPO data 2026-07-13
</commit_message>
<xml_diff>
--- a/IPO_Rawdata_master.xlsx
+++ b/IPO_Rawdata_master.xlsx
@@ -105177,13 +105177,23 @@
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="N44" t="n">
+        <v>900000</v>
+      </c>
+      <c r="O44" t="n">
+        <v>20700</v>
+      </c>
       <c r="P44" t="n">
         <v>1</v>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
+      <c r="Q44" t="n">
+        <v>900000</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>07-01~07-02</t>
+        </is>
+      </c>
       <c r="S44" t="inlineStr">
         <is>
           <t>2026-07-06</t>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-24
</commit_message>
<xml_diff>
--- a/IPO_Rawdata_master.xlsx
+++ b/IPO_Rawdata_master.xlsx
@@ -101841,7 +101841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -105133,12 +105133,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>미상장(납입완료)</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>에이치엘지노믹스</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -105147,7 +105147,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>248.4</v>
+        <v>551.48</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -105155,16 +105155,16 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>248.4</v>
+        <v>496.33</v>
       </c>
       <c r="H44" t="n">
-        <v>12.793</v>
+        <v>12.757</v>
       </c>
       <c r="I44" t="n">
-        <v>1.863</v>
+        <v>3.722</v>
       </c>
       <c r="J44" t="n">
-        <v>14.656</v>
+        <v>16.479</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -105178,23 +105178,165 @@
       </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="n">
+        <v>1731367</v>
+      </c>
+      <c r="O44" t="n">
+        <v>21500</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0.899996</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>1923750</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>07-13~07-14</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>에이치엘지노믹스</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>551.48</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>IBK</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>55.15</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.417</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1.831</v>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>공동주관</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="n">
+        <v>192383</v>
+      </c>
+      <c r="O45" t="n">
+        <v>21500</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0.100004</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1923750</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>07-13~07-14</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>미상장(납입완료)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>레메디</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>248.4</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>248.4</v>
+      </c>
+      <c r="H46" t="n">
+        <v>12.793</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.863</v>
+      </c>
+      <c r="J46" t="n">
+        <v>14.656</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>대표</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="n">
         <v>900000</v>
       </c>
-      <c r="O44" t="n">
+      <c r="O46" t="n">
         <v>20700</v>
       </c>
-      <c r="P44" t="n">
+      <c r="P46" t="n">
         <v>1</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="Q46" t="n">
         <v>900000</v>
       </c>
-      <c r="R44" t="inlineStr">
+      <c r="R46" t="inlineStr">
         <is>
           <t>07-01~07-02</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr">
+      <c r="S46" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>

</xml_diff>